<commit_message>
corrigindo divergência de preços
</commit_message>
<xml_diff>
--- a/02-Referencias/Rateio_APOIO_Março.xlsx
+++ b/02-Referencias/Rateio_APOIO_Março.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -448,250 +448,282 @@
         <v>-28963.82</v>
       </c>
       <c r="C2" t="n">
-        <v>0.5891316295517942</v>
+        <v>0.4730951204126361</v>
       </c>
       <c r="D2" t="n">
-        <v>58.91316295517942</v>
+        <v>47.30951204126362</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DESPESAS DE VIAGEM</t>
+          <t>HONORÁRIOS PJ</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-5956.42</v>
+        <v>-10000</v>
       </c>
       <c r="C3" t="n">
-        <v>0.121155131501815</v>
+        <v>0.1633400291855964</v>
       </c>
       <c r="D3" t="n">
-        <v>12.1155131501815</v>
+        <v>16.33400291855964</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BOLSA ESTAGIO</t>
+          <t>DESPESAS DE VIAGEM</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-5000</v>
+        <v>-5956.42</v>
       </c>
       <c r="C4" t="n">
-        <v>0.101701300027378</v>
+        <v>0.09729218166416703</v>
       </c>
       <c r="D4" t="n">
-        <v>10.1701300027378</v>
+        <v>9.729218166416704</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>EVENTOS ENDOMARKETING</t>
+          <t>BOLSA ESTAGIO</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-1907.89</v>
+        <v>-5000</v>
       </c>
       <c r="C5" t="n">
-        <v>0.03880697866184684</v>
+        <v>0.08167001459279821</v>
       </c>
       <c r="D5" t="n">
-        <v>3.880697866184684</v>
+        <v>8.16700145927982</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>HONORÁRIOS ADVOCATÍCIOS</t>
+          <t>EVENTOS ENDOMARKETING</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-1780</v>
+        <v>-2057.89</v>
       </c>
       <c r="C6" t="n">
-        <v>0.03620566280974656</v>
+        <v>0.03361358126607471</v>
       </c>
       <c r="D6" t="n">
-        <v>3.620566280974656</v>
+        <v>3.361358126607471</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ALUGUEL ADMINISTRATIVO</t>
+          <t>HONORÁRIOS ADVOCATÍCIOS</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-1670.31</v>
+        <v>-1780</v>
       </c>
       <c r="C7" t="n">
-        <v>0.03397453968974595</v>
+        <v>0.02907452519503616</v>
       </c>
       <c r="D7" t="n">
-        <v>3.397453968974594</v>
+        <v>2.907452519503616</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TELECOMUNICAÇÕES</t>
+          <t>ALUGUEL DE FUNCIONÁRIO</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-1106.02</v>
+        <v>-1750</v>
       </c>
       <c r="C8" t="n">
-        <v>0.02249673437125612</v>
+        <v>0.02858450510747938</v>
       </c>
       <c r="D8" t="n">
-        <v>2.249673437125612</v>
+        <v>2.858450510747938</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>DESPESAS BANCARIAS</t>
+          <t>ALUGUEL ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-697.4300000000001</v>
+        <v>-1670.31</v>
       </c>
       <c r="C9" t="n">
-        <v>0.01418590753561885</v>
+        <v>0.02728284841489936</v>
       </c>
       <c r="D9" t="n">
-        <v>1.418590753561885</v>
+        <v>2.728284841489935</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>INTERNET</t>
+          <t>TELECOMUNICAÇÕES</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>-589.71</v>
+        <v>-1106.02</v>
       </c>
       <c r="C10" t="n">
-        <v>0.01199485472782902</v>
+        <v>0.01806573390798534</v>
       </c>
       <c r="D10" t="n">
-        <v>1.199485472782901</v>
+        <v>1.806573390798534</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ALIMENTAÇÃO DO TRABALHADOR</t>
+          <t>DESPESAS BANCARIAS</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>-455.8</v>
+        <v>-697.4300000000001</v>
       </c>
       <c r="C11" t="n">
-        <v>0.009271090510495777</v>
+        <v>0.01139182365549105</v>
       </c>
       <c r="D11" t="n">
-        <v>0.9271090510495776</v>
+        <v>1.139182365549105</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ELETRÔNICOS</t>
+          <t>INTERNET</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-300</v>
+        <v>-589.71</v>
       </c>
       <c r="C12" t="n">
-        <v>0.006102078001642679</v>
+        <v>0.009632324861103807</v>
       </c>
       <c r="D12" t="n">
-        <v>0.6102078001642679</v>
+        <v>0.9632324861103807</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>SISTEMAS</t>
+          <t>ALIMENTAÇÃO DO TRABALHADOR</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>-296.57</v>
+        <v>-495.7</v>
       </c>
       <c r="C13" t="n">
-        <v>0.006032310909823898</v>
+        <v>0.008096765246730015</v>
       </c>
       <c r="D13" t="n">
-        <v>0.6032310909823898</v>
+        <v>0.8096765246730016</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ISS</t>
+          <t>SISTEMAS</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>-170.85</v>
+        <v>-415.07</v>
       </c>
       <c r="C14" t="n">
-        <v>0.003475133421935506</v>
+        <v>0.006779754591406551</v>
       </c>
       <c r="D14" t="n">
-        <v>0.3475133421935506</v>
+        <v>0.6779754591406552</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>MATERIAL DE LIMPEZA E HIGIENE</t>
+          <t>ELETRÔNICOS</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>-145.96</v>
+        <v>-300</v>
       </c>
       <c r="C15" t="n">
-        <v>0.002968864350399218</v>
+        <v>0.004900200875567893</v>
       </c>
       <c r="D15" t="n">
-        <v>0.2968864350399218</v>
+        <v>0.4900200875567893</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>TAXAS E LICENÇAS</t>
+          <t>ISS</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>-92.8</v>
+        <v>-170.85</v>
       </c>
       <c r="C16" t="n">
-        <v>0.001887576128508135</v>
+        <v>0.002790664398635915</v>
       </c>
       <c r="D16" t="n">
-        <v>0.1887576128508135</v>
+        <v>0.2790664398635915</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>MATERIAL DE LIMPEZA E HIGIENE</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>-145.96</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0.002384111065992965</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.2384111065992965</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>TAXAS E LICENÇAS</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>-92.8</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0.001515795470842335</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.1515795470842335</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>BRINDES</t>
         </is>
       </c>
-      <c r="B17" t="n">
+      <c r="B19" t="n">
         <v>-30</v>
       </c>
-      <c r="C17" t="n">
-        <v>0.0006102078001642679</v>
-      </c>
-      <c r="D17" t="n">
-        <v>0.06102078001642679</v>
+      <c r="C19" t="n">
+        <v>0.0004900200875567893</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.04900200875567893</v>
       </c>
     </row>
   </sheetData>

</xml_diff>